<commit_message>
machine learning - pset 2 (LDA, QDA, logit, Naive Bayes)
</commit_message>
<xml_diff>
--- a/4_autumn_2026/investments/pset_4/ps4_question3-1.xlsx
+++ b/4_autumn_2026/investments/pset_4/ps4_question3-1.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10709"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ngormsen/Dropbox/Booth/Teaching booth/Investments 2019/Problem sets/PS3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jballesteros/Documents/git/uchicago-mpp/4_autumn_2026/investments/pset_4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73099C69-BF8E-784A-90AD-DBF9A34D5BE1}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB91270-C873-D94B-BCCA-1731EF8E62A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17480" yWindow="6020" windowWidth="25600" windowHeight="14620" tabRatio="500"/>
+    <workbookView xWindow="-4480" yWindow="-20980" windowWidth="38400" windowHeight="20980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test2.csv" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>Quarter</t>
   </si>
@@ -33,13 +46,45 @@
   <si>
     <t>Value</t>
   </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>stdev</t>
+  </si>
+  <si>
+    <t>market-small</t>
+  </si>
+  <si>
+    <t>market-value</t>
+  </si>
+  <si>
+    <t>small-value</t>
+  </si>
+  <si>
+    <t>correlation</t>
+  </si>
+  <si>
+    <t>covariance</t>
+  </si>
+  <si>
+    <t>variance</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -67,9 +112,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,15 +522,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
     <col min="2" max="2" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -498,7 +544,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>200801</v>
       </c>
@@ -511,8 +557,17 @@
       <c r="D3">
         <v>-0.44791999999999998</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="H3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>200802</v>
       </c>
@@ -525,8 +580,23 @@
       <c r="D4">
         <v>2.3300999999999999E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <f>AVERAGE(B3:B44)</f>
+        <v>9.8566447619047606E-2</v>
+      </c>
+      <c r="I4">
+        <f>AVERAGE(C3:C44)</f>
+        <v>0.1192016119047619</v>
+      </c>
+      <c r="J4">
+        <f>AVERAGE(D3:D44)</f>
+        <v>0.11545617619047618</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>200803</v>
       </c>
@@ -539,8 +609,23 @@
       <c r="D5">
         <v>-0.31953999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <f>STDEV(B3:B44)</f>
+        <v>0.32705741796524779</v>
+      </c>
+      <c r="I5">
+        <f t="shared" ref="I5:J5" si="0">STDEV(C3:C44)</f>
+        <v>0.41592850431744327</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>0.35371210800352726</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>200804</v>
       </c>
@@ -553,8 +638,23 @@
       <c r="D6">
         <v>-0.9335</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <f>H5^2</f>
+        <v>0.10696655464609478</v>
+      </c>
+      <c r="I6">
+        <f>I5^2</f>
+        <v>0.17299652070374544</v>
+      </c>
+      <c r="J6">
+        <f>J5^2</f>
+        <v>0.12511225534829892</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>200901</v>
       </c>
@@ -568,7 +668,7 @@
         <v>-0.27328000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>200902</v>
       </c>
@@ -581,8 +681,17 @@
       <c r="D8">
         <v>0.81715000000000004</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="H8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>200903</v>
       </c>
@@ -595,8 +704,23 @@
       <c r="D9">
         <v>0.55018999999999996</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <f>CORREL(B3:B44, C3:C44)</f>
+        <v>0.94690058584574099</v>
+      </c>
+      <c r="I9">
+        <f>CORREL(B3:B44, D3:D44)</f>
+        <v>0.96763163587708267</v>
+      </c>
+      <c r="J9">
+        <f>CORREL(C3:C44, D3:D44)</f>
+        <v>0.94856387882316728</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>200904</v>
       </c>
@@ -609,8 +733,23 @@
       <c r="D10">
         <v>0.21908</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10">
+        <f>_xlfn.COVARIANCE.S(B3:B44,C3:C44)</f>
+        <v>0.1288092564819536</v>
+      </c>
+      <c r="I10">
+        <f>_xlfn.COVARIANCE.S(B3:B44,D3:D44)</f>
+        <v>0.11193966144942893</v>
+      </c>
+      <c r="J10">
+        <f>_xlfn.COVARIANCE.S(C3:C44,D3:D44)</f>
+        <v>0.13955172000203836</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>201001</v>
       </c>
@@ -624,7 +763,7 @@
         <v>0.21770999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>201002</v>
       </c>
@@ -638,7 +777,7 @@
         <v>-0.37513999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>201003</v>
       </c>
@@ -652,7 +791,7 @@
         <v>0.52659</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>201004</v>
       </c>
@@ -666,7 +805,7 @@
         <v>0.52937999999999996</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>201101</v>
       </c>
@@ -680,7 +819,7 @@
         <v>0.26425999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>201102</v>
       </c>

</xml_diff>